<commit_message>
Update docs to reflect final installation and decisions
Update README, build log, wiring plan and BOM to reflect that the control box, MPU6050, rotary encoder and LED strips are permanently installed in the MR2. Clarifies that only firmware tuning (v2.2 and beyond) remains. Documents the decision to accept (not fix) the USB-power backfeed and the minor speaker noise, and notes the removed master switch and replacement of the specified buck converter with a repurposed USB charger module. Hardware BOM spreadsheet updated to match the current build.
</commit_message>
<xml_diff>
--- a/hardware/bom/MR2_Reactive_LEDs_System_BOM.xlsx
+++ b/hardware/bom/MR2_Reactive_LEDs_System_BOM.xlsx
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Not yet purchased</t>
+          <t>Not purchased — decided not to pursue</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Planned fix, not yet installed — see build log "USB Power Backfeed Discovered"</t>
+          <t>Would fix a known minor USB-power backfeed issue, but impact judged too small to be worth it — see build log</t>
         </is>
       </c>
     </row>

</xml_diff>